<commit_message>
update run group analysis
</commit_message>
<xml_diff>
--- a/inst/extdata/loa_template.xlsx
+++ b/inst/extdata/loa_template.xlsx
@@ -1,33 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://drcngo-my.sharepoint.com/personal/cd538_drc_ngo/Documents/Desktop/Projects/Analysis Kit/analysiskit/docs/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_2E9D3C1C6B7123A1257391AF085467D75A9CB660" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C8AF596-6AF6-4CF1-AE45-54FA90500C0C}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1605" windowWidth="29040" windowHeight="15720" tabRatio="677" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
-    <sheet name="readme" sheetId="1" r:id="rId1"/>
-    <sheet name="analysis" sheetId="2" r:id="rId2"/>
-    <sheet name="group_analysis" sheetId="3" r:id="rId3"/>
-    <sheet name="count_selections" sheetId="4" r:id="rId4"/>
-    <sheet name="count_combinations" sheetId="5" r:id="rId5"/>
-    <sheet name="count_exclusive_combinations" sheetId="6" r:id="rId6"/>
-    <sheet name="exclude_choices" sheetId="7" r:id="rId7"/>
-    <sheet name="settings" sheetId="8" r:id="rId8"/>
+    <sheet name="readme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="analysis" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="group_analysis" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="count_selections" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="count_combinations" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="count_exclusive_combinations" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="exclude_choices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="settings" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
   <si>
     <t>Analysis Kit — List of Analysis workbook</t>
   </si>
@@ -387,13 +380,74 @@
   </si>
   <si>
     <t>Other choices only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">count_combinations_other_multiple_label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other multiple selection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">count_combinations_heading</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Choice combinations (of those who selected more than one choice)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">count_exclusive_combinations_heading</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single choices (of those who selected only one choice)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">count_exclusive_combinations_only_suffix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">" only"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">count_exclusive_combinations_other_label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other single selection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The two combination blocks split one base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">count_combinations reports the respondents who selected MORE THAN ONE choice:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Economic + Conflict only", "Economic + Conflict + Other", "Economic + Other".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">count_exclusive_combinations reports those who selected EXACTLY ONE choice:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Economic only", "Conflict only", "Other single selection".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both sit on the same denominator - everyone who answered and selected at least</t>
+  </si>
+  <si>
+    <t xml:space="preserve">one choice - so the two blocks TOGETHER add to 100%, while each block on its</t>
+  </si>
+  <si>
+    <t xml:space="preserve">own adds to the share of the sample it covers. Fill in both sheets to get both.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A respondent who answered but has no choice recorded is outside both blocks;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analysis Kit reports how many that is per question.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -402,8 +456,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="13"/>
+      <color rgb="FF003D58"/>
+      <name val="Arial"/>
       <b/>
-      <sz val="13"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF003D58"/>
       <name val="Arial"/>
     </font>
@@ -411,18 +470,13 @@
       <sz val="10"/>
       <color rgb="FF003D58"/>
       <name val="Arial"/>
+      <b/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF003D58"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <b/>
     </font>
   </fonts>
   <fills count="4">
@@ -455,7 +509,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -464,7 +518,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -766,269 +819,272 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <tabColor rgb="FF00A2A5"/>
   </sheetPr>
-  <dimension ref="A1:A50"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="92" customWidth="1"/>
+    <col min="1" max="1" width="92" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" ht="16.8" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" s="2"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5">
       <c r="A5" s="2"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9">
       <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10">
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11">
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="12">
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13">
       <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="14">
       <c r="A14" s="2"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="15">
       <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="16">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18">
       <c r="A18" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19">
       <c r="A19" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20">
       <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21">
       <c r="A21" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22">
       <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23">
       <c r="A23" s="2"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24">
       <c r="A24" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25">
       <c r="A25" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26">
       <c r="A26" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27">
       <c r="A27" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28">
       <c r="A28" s="2"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29">
       <c r="A29" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30">
       <c r="A30" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31">
       <c r="A31" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="32">
       <c r="A32" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="33">
       <c r="A33" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="34">
       <c r="A34" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="35">
       <c r="A35" s="2"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="36">
       <c r="A36" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="37">
       <c r="A37" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="38">
       <c r="A38" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="39">
       <c r="A39" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="40">
       <c r="A40" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="41">
       <c r="A41" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="42">
       <c r="A42" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="43">
       <c r="A43" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A44" s="2"/>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="45">
       <c r="A45" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="46">
       <c r="A46" s="2"/>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="47">
       <c r="A47" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="48">
       <c r="A48" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="49">
       <c r="A49" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="50">
       <c r="A50" s="2" t="s">
         <v>41</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="10" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="26" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" s="4" t="s">
         <v>42</v>
       </c>
@@ -1048,11 +1104,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="2" t="s">
         <v>49</v>
       </c>
       <c r="C2" s="2"/>
@@ -1062,11 +1118,11 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="2" t="s">
         <v>52</v>
       </c>
       <c r="C3" s="2"/>
@@ -1076,14 +1132,14 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="A4" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="2" t="n">
         <v>0.95</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -1092,11 +1148,11 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5">
       <c r="A5" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="2" t="s">
         <v>56</v>
       </c>
       <c r="C5" s="2"/>
@@ -1106,11 +1162,11 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6">
       <c r="A6" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="2" t="s">
         <v>56</v>
       </c>
       <c r="C6" s="2"/>
@@ -1122,20 +1178,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="36" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="1" max="1" width="36" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="10" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" s="4" t="s">
         <v>58</v>
       </c>
@@ -1146,7 +1203,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" s="2" t="s">
         <v>49</v>
       </c>
@@ -1157,7 +1214,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" s="5" t="s">
         <v>62</v>
       </c>
@@ -1168,7 +1225,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="A4" s="5" t="s">
         <v>64</v>
       </c>
@@ -1179,7 +1236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5">
       <c r="A5" s="5" t="s">
         <v>66</v>
       </c>
@@ -1190,7 +1247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6">
       <c r="A6" s="5" t="s">
         <v>68</v>
       </c>
@@ -1203,19 +1260,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="10" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" s="4" t="s">
         <v>43</v>
       </c>
@@ -1223,7 +1281,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" s="2" t="s">
         <v>52</v>
       </c>
@@ -1233,21 +1291,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="56" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="56" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="10" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" s="4" t="s">
         <v>43</v>
       </c>
@@ -1261,7 +1320,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" s="2" t="s">
         <v>52</v>
       </c>
@@ -1275,7 +1334,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" s="2" t="s">
         <v>52</v>
       </c>
@@ -1291,21 +1350,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="56" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="56" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="10" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" s="4" t="s">
         <v>43</v>
       </c>
@@ -1319,7 +1379,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" s="2" t="s">
         <v>52</v>
       </c>
@@ -1333,7 +1393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" s="2" t="s">
         <v>52</v>
       </c>
@@ -1349,19 +1409,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="1" max="1" width="32" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="10" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" s="4" t="s">
         <v>70</v>
       </c>
@@ -1369,7 +1430,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" s="2" t="s">
         <v>76</v>
       </c>
@@ -1377,7 +1438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" s="2" t="s">
         <v>77</v>
       </c>
@@ -1387,19 +1448,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="32" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1">
       <c r="A1" s="4" t="s">
         <v>78</v>
       </c>
@@ -1407,7 +1469,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2">
       <c r="A2" s="2" t="s">
         <v>80</v>
       </c>
@@ -1415,7 +1477,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3">
       <c r="A3" s="2" t="s">
         <v>82</v>
       </c>
@@ -1423,7 +1485,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4">
       <c r="A4" s="2" t="s">
         <v>84</v>
       </c>
@@ -1431,7 +1493,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5">
       <c r="A5" s="2" t="s">
         <v>85</v>
       </c>
@@ -1439,7 +1501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6">
       <c r="A6" s="2" t="s">
         <v>86</v>
       </c>
@@ -1447,25 +1509,25 @@
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7">
       <c r="A7" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B7" s="2"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8">
       <c r="A8" s="2" t="s">
         <v>89</v>
       </c>
       <c r="B8" s="2"/>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9">
       <c r="A9" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B9" s="2"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10">
       <c r="A10" s="2" t="s">
         <v>91</v>
       </c>
@@ -1473,7 +1535,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11">
       <c r="A11" s="2" t="s">
         <v>92</v>
       </c>
@@ -1481,7 +1543,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12">
       <c r="A12" s="2" t="s">
         <v>94</v>
       </c>
@@ -1489,7 +1551,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13">
       <c r="A13" s="2" t="s">
         <v>96</v>
       </c>
@@ -1497,7 +1559,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14">
       <c r="A14" s="2" t="s">
         <v>98</v>
       </c>
@@ -1505,7 +1567,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15">
       <c r="A15" s="2" t="s">
         <v>100</v>
       </c>
@@ -1513,7 +1575,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16">
       <c r="A16" s="2" t="s">
         <v>102</v>
       </c>
@@ -1521,7 +1583,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17">
       <c r="A17" s="2" t="s">
         <v>104</v>
       </c>
@@ -1529,7 +1591,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18">
       <c r="A18" s="2" t="s">
         <v>106</v>
       </c>
@@ -1537,15 +1599,15 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19">
       <c r="A19" s="2" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20" s="2" t="s">
         <v>109</v>
       </c>
@@ -1553,47 +1615,48 @@
         <v>110</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21">
       <c r="A21" s="2" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="22">
       <c r="A22" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="2" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23">
       <c r="A23" s="2" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="24">
       <c r="A24" s="2" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="25">
       <c r="A25" s="2" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>